<commit_message>
Bo sung Thang 10/2026: CBQL 10cv GV 12cv NV 8cv - Tong 30 cong viec giai doan T5-T10/2026 - Danh gia Thang 10 (kiem tra giua ky I)
</commit_message>
<xml_diff>
--- a/public/downloads/Import_cong_viec_GV.xlsx
+++ b/public/downloads/Import_cong_viec_GV.xlsx
@@ -520,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:L199"/>
+  <dimension ref="A2:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1534,736 +1534,413 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="9" t="n"/>
-      <c r="B36" s="10" t="n"/>
-      <c r="C36" s="10" t="n"/>
-      <c r="D36" s="9" t="n"/>
-      <c r="E36" s="9" t="n"/>
-      <c r="F36" s="9" t="n"/>
-      <c r="G36" s="9" t="n"/>
-      <c r="H36" s="10" t="n"/>
+      <c r="A36" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>Thực hiện giảng dạy đảm bảo tiến độ chương trình tháng 10, soạn bài đầy đủ theo CV 5512, sử dụng đồ dùng dạy học và ứng dụng CNTT hiệu quả</t>
+        </is>
+      </c>
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>N2_1115 - Kế hoạch triển khai hoạt động chuyên môn</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F36" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G36" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H36" s="10" t="inlineStr">
+        <is>
+          <t>Giáo án điện tử tháng 10 và sổ ghi đầu bài đảm bảo tiến độ</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="9" t="n"/>
-      <c r="B37" s="10" t="n"/>
-      <c r="C37" s="10" t="n"/>
-      <c r="D37" s="9" t="n"/>
-      <c r="E37" s="9" t="n"/>
-      <c r="F37" s="9" t="n"/>
-      <c r="G37" s="9" t="n"/>
-      <c r="H37" s="10" t="n"/>
+      <c r="A37" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>Ra đề, coi thi, chấm bài kiểm tra giữa học kỳ I theo ma trận đặc tả đã xây dựng; nhập điểm đầy đủ lên VnEdu đúng hạn</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>N1_564 - Quản lý dữ liệu của các Kỳ thi</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F37" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G37" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H37" s="10" t="inlineStr">
+        <is>
+          <t>Đề kiểm tra giữa HKI có ma trận, bảng điểm cập nhật VnEdu</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="9" t="n"/>
-      <c r="B38" s="10" t="n"/>
-      <c r="C38" s="10" t="n"/>
-      <c r="D38" s="9" t="n"/>
-      <c r="E38" s="9" t="n"/>
-      <c r="F38" s="9" t="n"/>
-      <c r="G38" s="9" t="n"/>
-      <c r="H38" s="10" t="n"/>
+      <c r="A38" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>Thực hiện sinh hoạt tổ chuyên môn tháng 10 theo chủ đề đổi mới phương pháp dạy học, nghiên cứu bài học và ứng dụng AI</t>
+        </is>
+      </c>
+      <c r="C38" s="10" t="inlineStr">
+        <is>
+          <t>N2_1115 - Kế hoạch triển khai hoạt động chuyên môn</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F38" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G38" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H38" s="10" t="inlineStr">
+        <is>
+          <t>Biên bản sinh hoạt tổ chuyên môn tháng 10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="9" t="n"/>
-      <c r="B39" s="10" t="n"/>
-      <c r="C39" s="10" t="n"/>
-      <c r="D39" s="9" t="n"/>
-      <c r="E39" s="9" t="n"/>
-      <c r="F39" s="9" t="n"/>
-      <c r="G39" s="9" t="n"/>
-      <c r="H39" s="10" t="n"/>
+      <c r="A39" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>Dự giờ đồng nghiệp đạt ít nhất 2 tiết/tháng, ghi nhận xét cụ thể và trao đổi phương pháp dạy học sau tiết dự giờ</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>N2_1115 - Kế hoạch triển khai hoạt động chuyên môn</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F39" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G39" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H39" s="10" t="inlineStr">
+        <is>
+          <t>Sổ dự giờ tháng 10 có nhận xét chi tiết và chữ ký</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="9" t="n"/>
-      <c r="B40" s="10" t="n"/>
-      <c r="C40" s="10" t="n"/>
-      <c r="D40" s="9" t="n"/>
-      <c r="E40" s="9" t="n"/>
-      <c r="F40" s="9" t="n"/>
-      <c r="G40" s="9" t="n"/>
-      <c r="H40" s="10" t="n"/>
+      <c r="A40" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>Tiếp tục bồi dưỡng học sinh giỏi môn phụ trách; tổ chức phụ đạo học sinh yếu kém đầu năm theo kế hoạch đã lập</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N2_1108 - Tổ chức kỳ thi chọn Đội tuyển tham dự kỳ thi chọn học sinh giỏi quốc gia THPT năm học 2026 - 2027 (tổ chức ra đề, coi thi, chấm </t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F40" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G40" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H40" s="10" t="inlineStr">
+        <is>
+          <t>Sổ bồi dưỡng HSG và danh sách học sinh tham gia phụ đạo tháng 10</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="9" t="n"/>
-      <c r="B41" s="10" t="n"/>
-      <c r="C41" s="10" t="n"/>
-      <c r="D41" s="9" t="n"/>
-      <c r="E41" s="9" t="n"/>
-      <c r="F41" s="9" t="n"/>
-      <c r="G41" s="9" t="n"/>
-      <c r="H41" s="10" t="n"/>
+      <c r="A41" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>Theo dõi, đánh giá nền nếp lớp chủ nhiệm tháng 10; tổ chức sinh hoạt lớp, họp lớp phân tích kết quả kiểm tra giữa kỳ</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>N1_565 - Quản lý, cập nhật cơ sở dữ liệu học sinh</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F41" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G41" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H41" s="10" t="inlineStr">
+        <is>
+          <t>Sổ chủ nhiệm tháng 10/2026 và biên bản sinh hoạt lớp</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="9" t="n"/>
-      <c r="B42" s="10" t="n"/>
-      <c r="C42" s="10" t="n"/>
-      <c r="D42" s="9" t="n"/>
-      <c r="E42" s="9" t="n"/>
-      <c r="F42" s="9" t="n"/>
-      <c r="G42" s="9" t="n"/>
-      <c r="H42" s="10" t="n"/>
+      <c r="A42" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>Thực hiện kiểm tra đánh giá thường xuyên đúng kế hoạch; chấm bài, trả bài, nhận xét cụ thể và vào điểm VnEdu kịp thời</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>N1_564 - Quản lý dữ liệu của các Kỳ thi</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="E42" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F42" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G42" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H42" s="10" t="inlineStr">
+        <is>
+          <t>Điểm kiểm tra thường xuyên tháng 10 cập nhật trên VnEdu</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="9" t="n"/>
-      <c r="B43" s="10" t="n"/>
-      <c r="C43" s="10" t="n"/>
-      <c r="D43" s="9" t="n"/>
-      <c r="E43" s="9" t="n"/>
-      <c r="F43" s="9" t="n"/>
-      <c r="G43" s="9" t="n"/>
-      <c r="H43" s="10" t="n"/>
+      <c r="A43" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>Đăng ký và tham gia tiết dạy mẫu, tiết dạy tốt chào mừng Ngày Nhà giáo Việt Nam 20/11; đăng ký thi giáo viên dạy giỏi cấp trường</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>N3_658 - Thẩm định hồ sơ và tham mưu công tác sáng kiến, đề tài nghiên cứu khoa học; các cuộc thi về công tác học sinh sinh viên; hồ sơ b</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>20/10/2026</t>
+        </is>
+      </c>
+      <c r="E43" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F43" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G43" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H43" s="10" t="inlineStr">
+        <is>
+          <t>Phiếu đăng ký thi GV dạy giỏi và đề cương tiết dạy mẫu</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="9" t="n"/>
-      <c r="B44" s="10" t="n"/>
-      <c r="C44" s="10" t="n"/>
-      <c r="D44" s="9" t="n"/>
-      <c r="E44" s="9" t="n"/>
-      <c r="F44" s="9" t="n"/>
-      <c r="G44" s="9" t="n"/>
-      <c r="H44" s="10" t="n"/>
+      <c r="A44" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t>Triển khai các nội dung bồi dưỡng thường xuyên tháng 10 theo kế hoạch cá nhân đã đăng ký; ghi nhật ký bồi dưỡng đầy đủ</t>
+        </is>
+      </c>
+      <c r="C44" s="10" t="inlineStr">
+        <is>
+          <t>N3_652 - Xây dựng Kế hoạch đào tạo, bồi dưỡng công chức, viên chức</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="E44" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F44" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G44" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H44" s="10" t="inlineStr">
+        <is>
+          <t>Nhật ký tự bồi dưỡng thường xuyên tháng 10/2026</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="9" t="n"/>
-      <c r="B45" s="10" t="n"/>
-      <c r="C45" s="10" t="n"/>
-      <c r="D45" s="9" t="n"/>
-      <c r="E45" s="9" t="n"/>
-      <c r="F45" s="9" t="n"/>
-      <c r="G45" s="9" t="n"/>
-      <c r="H45" s="10" t="n"/>
+      <c r="A45" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>Tham gia đầy đủ các buổi họp tổ chuyên môn, họp Hội đồng sư phạm tháng 10; hoàn thành phiếu đánh giá kết quả tháng 9</t>
+        </is>
+      </c>
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>N1_611 - Tổ chức, điều hành, đánh giá kết quả thực hiện nhiệm vụ của công chức thuộc phòng</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F45" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G45" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H45" s="10" t="inlineStr">
+        <is>
+          <t>Phiếu đánh giá kết quả thực hiện nhiệm vụ tháng 9/2026 có xác nhận TCM</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="9" t="n"/>
-      <c r="B46" s="10" t="n"/>
-      <c r="C46" s="10" t="n"/>
-      <c r="D46" s="9" t="n"/>
-      <c r="E46" s="9" t="n"/>
-      <c r="F46" s="9" t="n"/>
-      <c r="G46" s="9" t="n"/>
-      <c r="H46" s="10" t="n"/>
+      <c r="A46" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>Rà soát, cập nhật hồ sơ chuyên môn cá nhân: giáo án, kế hoạch dạy học, sổ ghi điểm theo đúng quy định của Sở GD&amp;ĐT</t>
+        </is>
+      </c>
+      <c r="C46" s="10" t="inlineStr">
+        <is>
+          <t>N2_1115 - Kế hoạch triển khai hoạt động chuyên môn</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="E46" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F46" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G46" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H46" s="10" t="inlineStr">
+        <is>
+          <t>Hồ sơ chuyên môn đầy đủ: giáo án, kế hoạch dạy học, sổ điểm</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="9" t="n"/>
-      <c r="B47" s="10" t="n"/>
-      <c r="C47" s="10" t="n"/>
-      <c r="D47" s="9" t="n"/>
-      <c r="E47" s="9" t="n"/>
-      <c r="F47" s="9" t="n"/>
-      <c r="G47" s="9" t="n"/>
-      <c r="H47" s="10" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="9" t="n"/>
-      <c r="B48" s="10" t="n"/>
-      <c r="C48" s="10" t="n"/>
-      <c r="D48" s="9" t="n"/>
-      <c r="E48" s="9" t="n"/>
-      <c r="F48" s="9" t="n"/>
-      <c r="G48" s="9" t="n"/>
-      <c r="H48" s="10" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="9" t="n"/>
-      <c r="B49" s="10" t="n"/>
-      <c r="C49" s="10" t="n"/>
-      <c r="D49" s="9" t="n"/>
-      <c r="E49" s="9" t="n"/>
-      <c r="F49" s="9" t="n"/>
-      <c r="G49" s="9" t="n"/>
-      <c r="H49" s="10" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="9" t="n"/>
-      <c r="B50" s="10" t="n"/>
-      <c r="C50" s="10" t="n"/>
-      <c r="D50" s="9" t="n"/>
-      <c r="E50" s="9" t="n"/>
-      <c r="F50" s="9" t="n"/>
-      <c r="G50" s="9" t="n"/>
-      <c r="H50" s="10" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="9" t="n"/>
-      <c r="B51" s="10" t="n"/>
-      <c r="C51" s="10" t="n"/>
-      <c r="D51" s="9" t="n"/>
-      <c r="E51" s="9" t="n"/>
-      <c r="F51" s="9" t="n"/>
-      <c r="G51" s="9" t="n"/>
-      <c r="H51" s="10" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="9" t="n"/>
-      <c r="B52" s="10" t="n"/>
-      <c r="C52" s="10" t="n"/>
-      <c r="D52" s="9" t="n"/>
-      <c r="E52" s="9" t="n"/>
-      <c r="F52" s="9" t="n"/>
-      <c r="G52" s="9" t="n"/>
-      <c r="H52" s="10" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="9" t="n"/>
-      <c r="B53" s="10" t="n"/>
-      <c r="C53" s="10" t="n"/>
-      <c r="D53" s="9" t="n"/>
-      <c r="E53" s="9" t="n"/>
-      <c r="F53" s="9" t="n"/>
-      <c r="G53" s="9" t="n"/>
-      <c r="H53" s="10" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="9" t="n"/>
-      <c r="B54" s="10" t="n"/>
-      <c r="C54" s="10" t="n"/>
-      <c r="D54" s="9" t="n"/>
-      <c r="E54" s="9" t="n"/>
-      <c r="F54" s="9" t="n"/>
-      <c r="G54" s="9" t="n"/>
-      <c r="H54" s="10" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="9" t="n"/>
-      <c r="B55" s="10" t="n"/>
-      <c r="C55" s="10" t="n"/>
-      <c r="D55" s="9" t="n"/>
-      <c r="E55" s="9" t="n"/>
-      <c r="F55" s="9" t="n"/>
-      <c r="G55" s="9" t="n"/>
-      <c r="H55" s="10" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="9" t="n"/>
-      <c r="B56" s="10" t="n"/>
-      <c r="C56" s="10" t="n"/>
-      <c r="D56" s="9" t="n"/>
-      <c r="E56" s="9" t="n"/>
-      <c r="F56" s="9" t="n"/>
-      <c r="G56" s="9" t="n"/>
-      <c r="H56" s="10" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="9" t="n"/>
-      <c r="B57" s="10" t="n"/>
-      <c r="C57" s="10" t="n"/>
-      <c r="D57" s="9" t="n"/>
-      <c r="E57" s="9" t="n"/>
-      <c r="F57" s="9" t="n"/>
-      <c r="G57" s="9" t="n"/>
-      <c r="H57" s="10" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="9" t="n"/>
-      <c r="B58" s="10" t="n"/>
-      <c r="C58" s="10" t="n"/>
-      <c r="D58" s="9" t="n"/>
-      <c r="E58" s="9" t="n"/>
-      <c r="F58" s="9" t="n"/>
-      <c r="G58" s="9" t="n"/>
-      <c r="H58" s="10" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="9" t="n"/>
-      <c r="B59" s="10" t="n"/>
-      <c r="C59" s="10" t="n"/>
-      <c r="D59" s="9" t="n"/>
-      <c r="E59" s="9" t="n"/>
-      <c r="F59" s="9" t="n"/>
-      <c r="G59" s="9" t="n"/>
-      <c r="H59" s="10" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="9" t="n"/>
-      <c r="B60" s="10" t="n"/>
-      <c r="C60" s="10" t="n"/>
-      <c r="D60" s="9" t="n"/>
-      <c r="E60" s="9" t="n"/>
-      <c r="F60" s="9" t="n"/>
-      <c r="G60" s="9" t="n"/>
-      <c r="H60" s="10" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="9" t="n"/>
-      <c r="B61" s="10" t="n"/>
-      <c r="C61" s="10" t="n"/>
-      <c r="D61" s="9" t="n"/>
-      <c r="E61" s="9" t="n"/>
-      <c r="F61" s="9" t="n"/>
-      <c r="G61" s="9" t="n"/>
-      <c r="H61" s="10" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="9" t="n"/>
-      <c r="B62" s="10" t="n"/>
-      <c r="C62" s="10" t="n"/>
-      <c r="D62" s="9" t="n"/>
-      <c r="E62" s="9" t="n"/>
-      <c r="F62" s="9" t="n"/>
-      <c r="G62" s="9" t="n"/>
-      <c r="H62" s="10" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="9" t="n"/>
-      <c r="B63" s="10" t="n"/>
-      <c r="C63" s="10" t="n"/>
-      <c r="D63" s="9" t="n"/>
-      <c r="E63" s="9" t="n"/>
-      <c r="F63" s="9" t="n"/>
-      <c r="G63" s="9" t="n"/>
-      <c r="H63" s="10" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="9" t="n"/>
-      <c r="B64" s="10" t="n"/>
-      <c r="C64" s="10" t="n"/>
-      <c r="D64" s="9" t="n"/>
-      <c r="E64" s="9" t="n"/>
-      <c r="F64" s="9" t="n"/>
-      <c r="G64" s="9" t="n"/>
-      <c r="H64" s="10" t="n"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="9" t="n"/>
-      <c r="B65" s="10" t="n"/>
-      <c r="C65" s="10" t="n"/>
-      <c r="D65" s="9" t="n"/>
-      <c r="E65" s="9" t="n"/>
-      <c r="F65" s="9" t="n"/>
-      <c r="G65" s="9" t="n"/>
-      <c r="H65" s="10" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="9" t="n"/>
-      <c r="B66" s="10" t="n"/>
-      <c r="C66" s="10" t="n"/>
-      <c r="D66" s="9" t="n"/>
-      <c r="E66" s="9" t="n"/>
-      <c r="F66" s="9" t="n"/>
-      <c r="G66" s="9" t="n"/>
-      <c r="H66" s="10" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="9" t="n"/>
-      <c r="B67" s="10" t="n"/>
-      <c r="C67" s="10" t="n"/>
-      <c r="D67" s="9" t="n"/>
-      <c r="E67" s="9" t="n"/>
-      <c r="F67" s="9" t="n"/>
-      <c r="G67" s="9" t="n"/>
-      <c r="H67" s="10" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="9" t="n"/>
-      <c r="B68" s="10" t="n"/>
-      <c r="C68" s="10" t="n"/>
-      <c r="D68" s="9" t="n"/>
-      <c r="E68" s="9" t="n"/>
-      <c r="F68" s="9" t="n"/>
-      <c r="G68" s="9" t="n"/>
-      <c r="H68" s="10" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="9" t="n"/>
-      <c r="B69" s="10" t="n"/>
-      <c r="C69" s="10" t="n"/>
-      <c r="D69" s="9" t="n"/>
-      <c r="E69" s="9" t="n"/>
-      <c r="F69" s="9" t="n"/>
-      <c r="G69" s="9" t="n"/>
-      <c r="H69" s="10" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="9" t="n"/>
-      <c r="B70" s="10" t="n"/>
-      <c r="C70" s="10" t="n"/>
-      <c r="D70" s="9" t="n"/>
-      <c r="E70" s="9" t="n"/>
-      <c r="F70" s="9" t="n"/>
-      <c r="G70" s="9" t="n"/>
-      <c r="H70" s="10" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="9" t="n"/>
-      <c r="B71" s="10" t="n"/>
-      <c r="C71" s="10" t="n"/>
-      <c r="D71" s="9" t="n"/>
-      <c r="E71" s="9" t="n"/>
-      <c r="F71" s="9" t="n"/>
-      <c r="G71" s="9" t="n"/>
-      <c r="H71" s="10" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="9" t="n"/>
-      <c r="B72" s="10" t="n"/>
-      <c r="C72" s="10" t="n"/>
-      <c r="D72" s="9" t="n"/>
-      <c r="E72" s="9" t="n"/>
-      <c r="F72" s="9" t="n"/>
-      <c r="G72" s="9" t="n"/>
-      <c r="H72" s="10" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="9" t="n"/>
-      <c r="B73" s="10" t="n"/>
-      <c r="C73" s="10" t="n"/>
-      <c r="D73" s="9" t="n"/>
-      <c r="E73" s="9" t="n"/>
-      <c r="F73" s="9" t="n"/>
-      <c r="G73" s="9" t="n"/>
-      <c r="H73" s="10" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="9" t="n"/>
-      <c r="B74" s="10" t="n"/>
-      <c r="C74" s="10" t="n"/>
-      <c r="D74" s="9" t="n"/>
-      <c r="E74" s="9" t="n"/>
-      <c r="F74" s="9" t="n"/>
-      <c r="G74" s="9" t="n"/>
-      <c r="H74" s="10" t="n"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="9" t="n"/>
-      <c r="B75" s="10" t="n"/>
-      <c r="C75" s="10" t="n"/>
-      <c r="D75" s="9" t="n"/>
-      <c r="E75" s="9" t="n"/>
-      <c r="F75" s="9" t="n"/>
-      <c r="G75" s="9" t="n"/>
-      <c r="H75" s="10" t="n"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="9" t="n"/>
-      <c r="B76" s="10" t="n"/>
-      <c r="C76" s="10" t="n"/>
-      <c r="D76" s="9" t="n"/>
-      <c r="E76" s="9" t="n"/>
-      <c r="F76" s="9" t="n"/>
-      <c r="G76" s="9" t="n"/>
-      <c r="H76" s="10" t="n"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="9" t="n"/>
-      <c r="B77" s="10" t="n"/>
-      <c r="C77" s="10" t="n"/>
-      <c r="D77" s="9" t="n"/>
-      <c r="E77" s="9" t="n"/>
-      <c r="F77" s="9" t="n"/>
-      <c r="G77" s="9" t="n"/>
-      <c r="H77" s="10" t="n"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="9" t="n"/>
-      <c r="B78" s="10" t="n"/>
-      <c r="C78" s="10" t="n"/>
-      <c r="D78" s="9" t="n"/>
-      <c r="E78" s="9" t="n"/>
-      <c r="F78" s="9" t="n"/>
-      <c r="G78" s="9" t="n"/>
-      <c r="H78" s="10" t="n"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="9" t="n"/>
-      <c r="B79" s="10" t="n"/>
-      <c r="C79" s="10" t="n"/>
-      <c r="D79" s="9" t="n"/>
-      <c r="E79" s="9" t="n"/>
-      <c r="F79" s="9" t="n"/>
-      <c r="G79" s="9" t="n"/>
-      <c r="H79" s="10" t="n"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="9" t="n"/>
-      <c r="B80" s="10" t="n"/>
-      <c r="C80" s="10" t="n"/>
-      <c r="D80" s="9" t="n"/>
-      <c r="E80" s="9" t="n"/>
-      <c r="F80" s="9" t="n"/>
-      <c r="G80" s="9" t="n"/>
-      <c r="H80" s="10" t="n"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="9" t="n"/>
-      <c r="B81" s="10" t="n"/>
-      <c r="C81" s="10" t="n"/>
-      <c r="D81" s="9" t="n"/>
-      <c r="E81" s="9" t="n"/>
-      <c r="F81" s="9" t="n"/>
-      <c r="G81" s="9" t="n"/>
-      <c r="H81" s="10" t="n"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="9" t="n"/>
-      <c r="B82" s="10" t="n"/>
-      <c r="C82" s="10" t="n"/>
-      <c r="D82" s="9" t="n"/>
-      <c r="E82" s="9" t="n"/>
-      <c r="F82" s="9" t="n"/>
-      <c r="G82" s="9" t="n"/>
-      <c r="H82" s="10" t="n"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="9" t="n"/>
-      <c r="B83" s="10" t="n"/>
-      <c r="C83" s="10" t="n"/>
-      <c r="D83" s="9" t="n"/>
-      <c r="E83" s="9" t="n"/>
-      <c r="F83" s="9" t="n"/>
-      <c r="G83" s="9" t="n"/>
-      <c r="H83" s="10" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="9" t="n"/>
-      <c r="B84" s="10" t="n"/>
-      <c r="C84" s="10" t="n"/>
-      <c r="D84" s="9" t="n"/>
-      <c r="E84" s="9" t="n"/>
-      <c r="F84" s="9" t="n"/>
-      <c r="G84" s="9" t="n"/>
-      <c r="H84" s="10" t="n"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="9" t="n"/>
-      <c r="B85" s="10" t="n"/>
-      <c r="C85" s="10" t="n"/>
-      <c r="D85" s="9" t="n"/>
-      <c r="E85" s="9" t="n"/>
-      <c r="F85" s="9" t="n"/>
-      <c r="G85" s="9" t="n"/>
-      <c r="H85" s="10" t="n"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="9" t="n"/>
-      <c r="B86" s="10" t="n"/>
-      <c r="C86" s="10" t="n"/>
-      <c r="D86" s="9" t="n"/>
-      <c r="E86" s="9" t="n"/>
-      <c r="F86" s="9" t="n"/>
-      <c r="G86" s="9" t="n"/>
-      <c r="H86" s="10" t="n"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="9" t="n"/>
-      <c r="B87" s="10" t="n"/>
-      <c r="C87" s="10" t="n"/>
-      <c r="D87" s="9" t="n"/>
-      <c r="E87" s="9" t="n"/>
-      <c r="F87" s="9" t="n"/>
-      <c r="G87" s="9" t="n"/>
-      <c r="H87" s="10" t="n"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="9" t="n"/>
-      <c r="B88" s="10" t="n"/>
-      <c r="C88" s="10" t="n"/>
-      <c r="D88" s="9" t="n"/>
-      <c r="E88" s="9" t="n"/>
-      <c r="F88" s="9" t="n"/>
-      <c r="G88" s="9" t="n"/>
-      <c r="H88" s="10" t="n"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="9" t="n"/>
-      <c r="B89" s="10" t="n"/>
-      <c r="C89" s="10" t="n"/>
-      <c r="D89" s="9" t="n"/>
-      <c r="E89" s="9" t="n"/>
-      <c r="F89" s="9" t="n"/>
-      <c r="G89" s="9" t="n"/>
-      <c r="H89" s="10" t="n"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="9" t="n"/>
-      <c r="B90" s="10" t="n"/>
-      <c r="C90" s="10" t="n"/>
-      <c r="D90" s="9" t="n"/>
-      <c r="E90" s="9" t="n"/>
-      <c r="F90" s="9" t="n"/>
-      <c r="G90" s="9" t="n"/>
-      <c r="H90" s="10" t="n"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="9" t="n"/>
-      <c r="B91" s="10" t="n"/>
-      <c r="C91" s="10" t="n"/>
-      <c r="D91" s="9" t="n"/>
-      <c r="E91" s="9" t="n"/>
-      <c r="F91" s="9" t="n"/>
-      <c r="G91" s="9" t="n"/>
-      <c r="H91" s="10" t="n"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="9" t="n"/>
-      <c r="B92" s="10" t="n"/>
-      <c r="C92" s="10" t="n"/>
-      <c r="D92" s="9" t="n"/>
-      <c r="E92" s="9" t="n"/>
-      <c r="F92" s="9" t="n"/>
-      <c r="G92" s="9" t="n"/>
-      <c r="H92" s="10" t="n"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="9" t="n"/>
-      <c r="B93" s="10" t="n"/>
-      <c r="C93" s="10" t="n"/>
-      <c r="D93" s="9" t="n"/>
-      <c r="E93" s="9" t="n"/>
-      <c r="F93" s="9" t="n"/>
-      <c r="G93" s="9" t="n"/>
-      <c r="H93" s="10" t="n"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="9" t="n"/>
-      <c r="B94" s="10" t="n"/>
-      <c r="C94" s="10" t="n"/>
-      <c r="D94" s="9" t="n"/>
-      <c r="E94" s="9" t="n"/>
-      <c r="F94" s="9" t="n"/>
-      <c r="G94" s="9" t="n"/>
-      <c r="H94" s="10" t="n"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="9" t="n"/>
-      <c r="B95" s="10" t="n"/>
-      <c r="C95" s="10" t="n"/>
-      <c r="D95" s="9" t="n"/>
-      <c r="E95" s="9" t="n"/>
-      <c r="F95" s="9" t="n"/>
-      <c r="G95" s="9" t="n"/>
-      <c r="H95" s="10" t="n"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="9" t="n"/>
-      <c r="B96" s="10" t="n"/>
-      <c r="C96" s="10" t="n"/>
-      <c r="D96" s="9" t="n"/>
-      <c r="E96" s="9" t="n"/>
-      <c r="F96" s="9" t="n"/>
-      <c r="G96" s="9" t="n"/>
-      <c r="H96" s="10" t="n"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="9" t="n"/>
-      <c r="B97" s="10" t="n"/>
-      <c r="C97" s="10" t="n"/>
-      <c r="D97" s="9" t="n"/>
-      <c r="E97" s="9" t="n"/>
-      <c r="F97" s="9" t="n"/>
-      <c r="G97" s="9" t="n"/>
-      <c r="H97" s="10" t="n"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="9" t="n"/>
-      <c r="B98" s="10" t="n"/>
-      <c r="C98" s="10" t="n"/>
-      <c r="D98" s="9" t="n"/>
-      <c r="E98" s="9" t="n"/>
-      <c r="F98" s="9" t="n"/>
-      <c r="G98" s="9" t="n"/>
-      <c r="H98" s="10" t="n"/>
-    </row>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
+      <c r="A47" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>Tiến hành bước đầu thu thập tài liệu, nghiên cứu và xây dựng đề cương chi tiết Sáng kiến kinh nghiệm năm học 2026 - 2027</t>
+        </is>
+      </c>
+      <c r="C47" s="10" t="inlineStr">
+        <is>
+          <t>N3_658 - Thẩm định hồ sơ và tham mưu công tác sáng kiến, đề tài nghiên cứu khoa học; các cuộc thi về công tác học sinh sinh viên; hồ sơ b</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="E47" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F47" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="G47" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H47" s="10" t="inlineStr">
+        <is>
+          <t>Đề cương SKKN năm học 2026-2027 đã hoàn thiện bước đầu</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A2:L2"/>

</xml_diff>